<commit_message>
Parallel grading verified working - 2 students graded simultaneously
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -44,6 +44,12 @@
   </x:si>
   <x:si>
     <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>dongnvhe172649</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hoangbsthe186345</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -409,10 +415,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F2"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.567768" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
@@ -460,6 +466,46 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D3" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Test run completed - applications starting and packets captured successfully
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -44,6 +44,12 @@
   </x:si>
   <x:si>
     <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>dongnvhe172649</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hoangbsthe186345</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -409,10 +415,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F2"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.567768" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
@@ -460,6 +466,46 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D3" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Fix golden server copying - students now getting marks (1/5 each)
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,7 +40,7 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>FAILED</x:t>
+    <x:t>PASSED</x:t>
   </x:si>
   <x:si>
     <x:t/>
@@ -420,7 +420,7 @@
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
@@ -457,7 +457,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>5</x:v>
@@ -477,7 +477,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>5</x:v>
@@ -497,7 +497,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
Fix flag matching - exact match with order normalization (not lenient subset)
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,13 +40,16 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
+    <x:t>FAILED</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>dongnvhe172649</x:t>
+  </x:si>
+  <x:si>
     <x:t>PASSED</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
@@ -457,7 +460,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>5</x:v>
@@ -474,7 +477,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>1</x:v>
@@ -488,13 +491,13 @@
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D4" s="0">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Fix TCP flag order to match reference implementation (PSH before ACK)
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -47,9 +47,6 @@
   </x:si>
   <x:si>
     <x:t>dongnvhe172649</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASSED</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
@@ -423,7 +420,7 @@
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
@@ -477,10 +474,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>5</x:v>
@@ -491,16 +488,16 @@
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
Cross-check complete: Parallel branch has server response issue
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,7 +40,7 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>FAILED</x:t>
+    <x:t>PASSED</x:t>
   </x:si>
   <x:si>
     <x:t/>
@@ -420,7 +420,7 @@
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
@@ -457,7 +457,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>5</x:v>
@@ -477,7 +477,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>5</x:v>
@@ -497,7 +497,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
Fix appsettings to use matching ports for direct mapping (8000:8000, 8001:8001)
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,7 +40,7 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>PASSED</x:t>
+    <x:t>FAILED</x:t>
   </x:si>
   <x:si>
     <x:t/>
@@ -420,7 +420,7 @@
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
@@ -457,7 +457,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>5</x:v>
@@ -477,7 +477,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>5</x:v>
@@ -497,7 +497,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
Parallel grading working - Docker image built, PortAllocator functional, applications starting
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,13 +40,16 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
+    <x:t>PASSED</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>dongnvhe172649</x:t>
+  </x:si>
+  <x:si>
     <x:t>FAILED</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
@@ -420,7 +423,7 @@
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
@@ -457,7 +460,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>5</x:v>
@@ -474,7 +477,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>0</x:v>
@@ -488,7 +491,7 @@
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>7</x:v>
@@ -497,7 +500,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
Fix cleanup to preserve container process - only kill application processes, not remove files
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,19 +40,28 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>PASSED</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
+    <x:t>FAILED</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No test kit for paper 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No test kit for paper 2</x:t>
   </x:si>
   <x:si>
     <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
-    <x:t>FAILED</x:t>
-  </x:si>
-  <x:si>
     <x:t>hoangbsthe186345</x:t>
+  </x:si>
+  <x:si>
+    <x:t>huynqhe172314</x:t>
+  </x:si>
+  <x:si>
+    <x:t>nhatnmhe186348</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -418,15 +427,15 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F4"/>
+  <x:dimension ref="A1:F9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6" s="1" customFormat="1">
@@ -460,10 +469,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
         <x:v>9</x:v>
@@ -471,22 +480,22 @@
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
       <x:c r="C3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D3" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
         <x:v>11</x:v>
-      </x:c>
-      <x:c r="D3" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E3" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -500,13 +509,113 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
         <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:6">
+      <x:c r="A7" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:6">
+      <x:c r="A8" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>11</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Parallel grading test complete - cuongnhhe=1/5, dongnvhe=0/5, hoangbsthe=4/5
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -43,25 +43,16 @@
     <x:t>FAILED</x:t>
   </x:si>
   <x:si>
-    <x:t>No test kit for paper 1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No test kit for paper 2</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
+    <x:t>PASSED</x:t>
+  </x:si>
+  <x:si>
     <x:t>hoangbsthe186345</x:t>
-  </x:si>
-  <x:si>
-    <x:t>huynqhe172314</x:t>
-  </x:si>
-  <x:si>
-    <x:t>nhatnmhe186348</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -427,15 +418,15 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F9"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20.282054" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6" s="1" customFormat="1">
@@ -472,7 +463,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
         <x:v>9</x:v>
@@ -480,22 +471,22 @@
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -506,116 +497,16 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
         <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:6">
-      <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:6">
-      <x:c r="A6" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:6">
-      <x:c r="A7" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D7" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F7" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:6">
-      <x:c r="A8" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D8" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:6">
-      <x:c r="A9" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D9" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="0" t="s">
-        <x:v>11</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Parallel grading working - cuongnhhe=1/5, dongnvhe=4/5, hoangbsthe=4/5 (TC1 timing issue affects all)
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/StudentsSolution.xlsx
+++ b/Submit/Results/StudentsSolution.xlsx
@@ -40,16 +40,13 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>FAILED</x:t>
+    <x:t>PASSED</x:t>
   </x:si>
   <x:si>
     <x:t/>
   </x:si>
   <x:si>
     <x:t>dongnvhe172649</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASSED</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
@@ -460,7 +457,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>5</x:v>
@@ -477,10 +474,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>5</x:v>
@@ -491,13 +488,13 @@
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="0">
         <x:v>4</x:v>

</xml_diff>